<commit_message>
Fill five-college UG/PG folders to 7 samples where found.
Keep original 论坛纷纭 texts. Add sourced extras into 学院名本科部 / 学院名研究生部 (max 7). GSTI undergraduate stays short because there is no regular bachelor programme. Refresh the first-person remainder workbook.

Co-authored-by: 36613453226Wallen <36613453226Wallen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/files/论坛风云/还剩多少第一人称视角の就读体验.xlsx
+++ b/files/论坛风云/还剩多少第一人称视角の就读体验.xlsx
@@ -624,7 +624,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -642,12 +642,12 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>（无）</t>
+          <t>北鼎-英美文学网面90.6</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>合格 0。还差 5 条独立就读自述才够业余印象门槛。</t>
+          <t>只有半合格。还差 5 条合格自述（门槛 5）。</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>0</v>
@@ -732,7 +732,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>考研论坛-2018俄语MTI复试现场</t>
+          <t>考研论坛-2018俄语MTI复试现场；听力室转载-2016俄语口译复试</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1072,14 +1072,14 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>01-本科-Insight-BFSU.txt；02-本科-Insight-BFSU.txt；03-本科-豆瓣小组.txt；04-本科-金榜教育转载问答.txt；05-本科-今日头条.txt</t>
+          <t>01-本科-Insight-BFSU.txt；02-本科-Insight-BFSU.txt；03-本科-豆瓣小组.txt；04-本科-金榜教育转载问答.txt；05-本科-今日头条.txt；09-本科-bigknow-转载问答.txt；10-本科-englang-保送经验转载.txt</t>
         </is>
       </c>
     </row>
@@ -1095,14 +1095,14 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>06-研究生部-北鼎教育.txt；07-研究生部-新祥旭考研.txt；08-研究生部-北鼎教育.txt</t>
+          <t>06-研究生部-北鼎教育.txt；07-研究生部-新祥旭考研.txt；08-研究生部-北鼎教育.txt；11-研究生部-北鼎教育.txt；12-研究生部-路灯在职研究生转载.txt；13-研究生部-北鼎教育.txt；14-研究生部-查字典考研网.txt</t>
         </is>
       </c>
     </row>
@@ -1118,14 +1118,14 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>01-本科-知乎.txt；02-本科-知乎.txt；03-本科-豆瓣小组.txt</t>
+          <t>01-本科-知乎.txt；02-本科-知乎.txt；03-本科-豆瓣小组.txt；08-本科建制-刀豆文库转载课程设置.txt；09-本科-俄语学院官网-毕业典礼发言.txt；10-本科-瀚博招生网问答转载.txt；11-本科-englang-保送说明.txt</t>
         </is>
       </c>
     </row>
@@ -1141,14 +1141,14 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>04-研究生部-考研论坛-kaoyan-com.txt；05-研究生部-Free考研-经验转载.txt；06-研究生部-新祥旭.txt；07-研究生部-瀚博招生网问答转载.txt</t>
+          <t>04-研究生部-考研论坛-kaoyan-com.txt；05-研究生部-Free考研-经验转载.txt；06-研究生部-新祥旭.txt；07-研究生部-瀚博招生网问答转载.txt；12-研究生部-听力室-学习网转载.txt；13-研究生部-新祥旭.txt；14-研究生部-北外校友会.txt</t>
         </is>
       </c>
     </row>
@@ -1164,14 +1164,14 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>01-本科建制-高翻学院官网推免方案.txt；02-本科-研究生入口-北鼎教育.txt</t>
+          <t>01-本科建制-高翻学院官网推免方案.txt；02-本科-研究生入口-北鼎教育.txt；09-本科建制-高翻学院官网-学院简介.txt</t>
         </is>
       </c>
     </row>
@@ -1187,14 +1187,14 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>03-研究生部-沪江英语访谈.txt；04-研究生部-高翻学院官网-新浪博客转载.txt；05-研究生部-高翻学院官网-毕业生专访.txt；06-研究生部-考研论坛-kaoyan-com.txt；07-研究生部-北鼎教育.txt；08-研究生部-写写帮转载.txt</t>
+          <t>03-研究生部-沪江英语访谈.txt；04-研究生部-高翻学院官网-新浪博客转载.txt；05-研究生部-高翻学院官网-毕业生专访.txt；06-研究生部-考研论坛-kaoyan-com.txt；07-研究生部-北鼎教育.txt；08-研究生部-写写帮转载.txt；10-研究生部-高翻学院官网-校友访谈.txt</t>
         </is>
       </c>
     </row>
@@ -1210,14 +1210,14 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>01-本科-研究生部-经管之家-人大经济论坛.txt；02-本科-经管之家.txt；08-本科-Reddit-r-ChinaLi.txt；09-本科-北外留学-iMAP-官网-学长学.txt</t>
+          <t>01-本科-研究生部-经管之家-人大经济论坛.txt；02-本科-经管之家.txt；08-本科-Reddit-r-ChinaLi.txt；09-本科-北外留学-iMAP-官网-学长学.txt；10-本科-高顿教育-ACCA.txt；11-本科-国际教育网.txt；12-本科建制-国际商学院官网.txt</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>03-研究生部-考研帮.txt；04-研究生部-查字典公务员网转载考研经验.txt；05-研究生部-经管之家.txt；06-研究生部-新祥旭.txt；07-研究生部-Reddit-r-ChinaLi.txt</t>
+          <t>03-研究生部-考研帮.txt；04-研究生部-查字典公务员网转载考研经验.txt；05-研究生部-经管之家.txt；06-研究生部-新祥旭.txt；07-研究生部-Reddit-r-ChinaLi.txt；13-研究生部-经管之家.txt；14-研究生部-文书帮.txt</t>
         </is>
       </c>
     </row>
@@ -1256,14 +1256,14 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>01-本科-中国青年报客户端-中青在线.txt；02-本科-教育问答转载.txt；03-本科-locks-wiki-转载旧论坛.txt；04-本科-知乎.txt</t>
+          <t>01-本科-中国青年报客户端-中青在线.txt；02-本科-教育问答转载.txt；03-本科-locks-wiki-转载旧论坛.txt；04-本科-知乎.txt；09-本科建制-国际关系学院官网-学院简介.txt；10-本科-北外国际交流合作处.txt；11-本科建制-掌上高考专业页.txt</t>
         </is>
       </c>
     </row>
@@ -1279,14 +1279,14 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>05-研究生部-考研帮.txt；06-研究生部-北鼎教育.txt；07-研究生部-北鼎教育.txt；08-研究生部-北鼎教育.txt</t>
+          <t>05-研究生部-考研帮.txt；06-研究生部-北鼎教育.txt；07-研究生部-北鼎教育.txt；08-研究生部-北鼎教育.txt；12-研究生部-Free考研转考研论坛.txt；13-研究生部-刀豆文库转载.txt；14-研究生部建制-国际关系学院官网-学院简介.txt</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1389,34 +1389,34 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>北鼎/新祥旭英文学硕</t>
+          <t>北鼎英美文学90.6、路灯跨考、查字典美国研究</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>考研机构上岸稿，不是读研日常</t>
+          <t>考研机构/转载站上岸稿，不是读研日常</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>俄语学院</t>
+          <t>高级翻译学院</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>豆瓣小语种辩护</t>
+          <t>张旭校友访谈（复语班作业否决项）</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>学校层，未写俄语学院</t>
+          <t>官网风采/出色个例，口径同尚姝辰</t>
         </is>
       </c>
     </row>
@@ -1433,19 +1433,19 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>新祥旭就业率100%</t>
+          <t>赵梦雪校友会采访</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>机构推销</t>
+          <t>本科在黑龙江大学；北外段是硕博出色个例</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>高级翻译学院</t>
+          <t>俄语学院</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1455,19 +1455,19 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>推免方案、保研指南</t>
+          <t>豆瓣小语种辩护</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>无普通本科就读对象</t>
+          <t>学校层，未写俄语学院</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>高级翻译学院</t>
+          <t>俄语学院</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>尚姝辰毕业生专访、李长栓访谈</t>
+          <t>新祥旭就业率100%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>官网风采/教师，不是学生论坛自述</t>
+          <t>机构推销</t>
         </is>
       </c>
     </row>
@@ -1494,61 +1494,61 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>北鼎法语口译在读</t>
+          <t>推免方案、保研指南</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>法语学院，不记入高翻</t>
+          <t>无普通本科就读对象</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>国际商学院</t>
+          <t>高级翻译学院</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>iMAP郑宽、国际本科评价</t>
+          <t>尚姝辰毕业生专访、李长栓访谈</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>留学项目≠统招</t>
+          <t>官网风采/教师，不是学生论坛自述</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>国际商学院</t>
+          <t>高级翻译学院</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>高顿倪子君双学位申哥大</t>
+          <t>北鼎法语口译在读</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ACCA机构学霸稿</t>
+          <t>法语学院，不记入高翻</t>
         </is>
       </c>
     </row>
@@ -1560,24 +1560,24 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>新祥旭MIB、Reddit申请帖</t>
+          <t>iMAP郑宽、国际本科评价</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>备考/申请，不是就读</t>
+          <t>留学项目≠统招</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>国际关系学院</t>
+          <t>国际商学院</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1587,34 +1587,34 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>中青报2021级外交学、国关优秀毕业生风采</t>
+          <t>高顿倪子君双学位申哥大</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>党媒/学院风采</t>
+          <t>ACCA机构学霸稿</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>国际关系学院</t>
+          <t>国际商学院</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Whever国关养老</t>
+          <t>新祥旭MIB、Reddit申请帖</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>俄语生外推，作者不在国关</t>
+          <t>备考/申请，不是就读</t>
         </is>
       </c>
     </row>
@@ -1626,59 +1626,103 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>北鼎复试/真题</t>
+          <t>中青报2021级外交学、国关优秀毕业生风采</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>机构备考</t>
+          <t>党媒/学院风采</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>校级未分院</t>
+          <t>国际关系学院</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>就读文章1 MouradBey、7 成就你的梦想</t>
+          <t>Whever国关养老</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>未写五院之一；第7篇是付费咨询</t>
+          <t>俄语生外推，作者不在国关</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>国际关系学院</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>研究生部</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>北鼎复试/真题</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>机构备考</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>校级未分院</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>就读文章1 MouradBey、7 成就你的梦想</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>未写五院之一；第7篇是付费咨询</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>他院</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>就读文章2 朝鲜语、3–4 MJC</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>亚洲学院/国新，不占五院格子</t>
         </is>
@@ -1746,7 +1790,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>高翻本科部不适用。续搜仍未找到英院研究生部、高翻研究生部的合格课堂日记。</t>
+          <t>高翻本科部不适用。续搜补了张旭复语班作业现场，但按出色个例不进合格格；英院研究生部仍无课堂日记。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill 自述权重+ with sourced first-person 在读 samples toward 7–10 per department.
Continue forum search into 论坛风云/自述权重+ rather than 论坛纷纭. Add verified first-person items (independent 合格 plus 约稿/考研 半合格), keep GSTI undergraduate as N/A, and record remaining gaps in the Excel workbook without inventing posts.

Co-authored-by: 36613453226Wallen <36613453226Wallen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/files/论坛风云/还剩多少第一人称视角の就读体验.xlsx
+++ b/files/论坛风云/还剩多少第一人称视角の就读体验.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'还剩多少'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'还剩多少'!$A$1:$M$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -496,12 +496,14 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -532,30 +534,40 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>本夹总条数</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>距每部下限7还差</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>合格独立叙述人数</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>还剩合格条数</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>还剩独立叙述者</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>够一般业余印象分析吗</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>已调用的自述类文章</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>缺口说明</t>
         </is>
@@ -579,30 +591,36 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>豆瓣-英院幸存者偏差；金榜转载-英专大二课表</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>合格 1 条 / 1 人。还差 4 条、2 个独立叙述者。</t>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>豆瓣-英院幸存者偏差；金榜转载-英专大二课表；Insight-康惠阳peer-pressure；Insight-吴旨瑨原著讨论；校友会征文-赵培85级精读听力</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>合格 1 条 / 1 人。还差 4 条、2 个独立叙述者。本夹 5 条，距每部 7 条还差 2。</t>
         </is>
       </c>
     </row>
@@ -624,30 +642,36 @@
         <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>北鼎-英美文学网面90.6</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>只有半合格。还差 5 条合格自述（门槛 5）。</t>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>北鼎-英美文学网面90.6；新祥旭-文学方向课全都上过；查字典-美国研究复试拟录取；路灯转载-跨考英语言文学复试；北鼎-工科跨考611</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>只有半合格。还差 5 条合格自述（门槛 5）。距每部 7 条还差 2。</t>
         </is>
       </c>
     </row>
@@ -669,30 +693,36 @@
         <v>2</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>就读文章5-Whever俄语后悔；就读文章6-Whever劝退俄语</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>合格 2 条 / 1 人。还差 3 条、2 个独立叙述者。</t>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>就读文章5-Whever俄语后悔；就读文章6-Whever劝退俄语；招生办-陆瑶一周俄语；豆瓣书评-08级东方俄语小白鼠</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>合格 2 条 / 1 人。还差 3 条、2 个独立叙述者。本夹 4 条，距每部 7 条还差 3。</t>
         </is>
       </c>
     </row>
@@ -714,30 +744,36 @@
         <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>考研论坛-2018俄语MTI复试现场；听力室转载-2016俄语口译复试</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>只有半合格。还差 5 条合格自述（门槛 5）。</t>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>考研论坛-2018俄语MTI复试现场；听力室转载-2016俄语口译复试；本科院校风采-刘岚普俄语笔译课；校友会-赵梦雪硕博口译练习</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>只有半合格。还差 5 条合格自述（门槛 5）。距每部 7 条还差 3。</t>
         </is>
       </c>
     </row>
@@ -770,17 +806,23 @@
       <c r="H6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>（无）</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>无普通本科就读对象。余量记 0，不要用保研文件凑数。</t>
         </is>
@@ -804,30 +846,36 @@
         <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>（无）</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>合格 0。还差 5 条独立就读自述才够业余印象门槛。</t>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>官网访谈-张旭复语班否决项；校友会-文苑李长栓200字reference；官网专访-尚姝辰研一口笔译；北鼎-研一依旧有演讲课；考研论坛-19高翻MA一战；李长栓文-匿名期末总结笔译助口译</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>只有半合格。还差 5 条合格自述（门槛 5）。距每部 7 条还差 1。</t>
         </is>
       </c>
     </row>
@@ -846,33 +894,39 @@
         <v>5</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>经管之家-曹渊国商大四考金专；经管之家-lu-llaby66北外金融本科推免</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>只有半合格。还差 5 条合格自述（门槛 5）。</t>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>经管之家-曹渊国商大四考金专；经管之家-lu-llaby66北外金融本科推免；豆瓣-国商会计财管培养方案</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>合格 1 条 / 1 人。还差 4 条、2 个独立叙述者。本夹 3 条，距每部 7 条还差 4。</t>
         </is>
       </c>
     </row>
@@ -894,30 +948,36 @@
         <v>0</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="J9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>查字典转载-金专入学后午餐会宿舍CFA；文书帮转载-国商学习两个多月</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>只有半合格。还差 5 条合格自述（门槛 5）。</t>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>查字典转载-金专入学后午餐会宿舍CFA；文书帮转载-国商学习两个多月；考研帮-生姜饼干金专复试；经管之家-simple_kaka国际商务拟录取</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>只有半合格。还差 5 条合格自述（门槛 5）。距每部 7 条还差 3。</t>
         </is>
       </c>
     </row>
@@ -939,30 +999,36 @@
         <v>1</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>转载-外交系在读双专业</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>合格 1 条 / 1 人。还差 4 条、2 个独立叙述者。</t>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>转载-外交系在读双专业；中青报-2021级外交学德语法语；灯塔留学-Anette外交学法语</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>合格 1 条 / 1 人。还差 4 条、2 个独立叙述者。本夹 3 条，距每部 7 条还差 4。</t>
         </is>
       </c>
     </row>
@@ -984,35 +1050,41 @@
         <v>0</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="J11" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>考研帮-wjb0911外交学毕业回看</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>只有半合格。还差 5 条合格自述（门槛 5）。</t>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>考研帮-wjb0911外交学毕业回看；Free考研-wjb0911外交学复试；刀豆文库-外交学复试跨专业；北鼎-国关无参考书真题体会；北鼎-外交学国际经济网面</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>只有半合格。还差 5 条合格自述（门槛 5）。距每部 7 条还差 2。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K11"/>
+  <autoFilter ref="A1:M11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1301,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1350,7 +1422,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>学院采访/学生组织约稿，出色个例</t>
+          <t>已进半合格。约稿出色个例，不充合格。</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1444,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>媒体成稿</t>
+          <t>媒体成稿，未进夹。</t>
         </is>
       </c>
     </row>
@@ -1384,24 +1456,24 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>北鼎英美文学90.6、路灯跨考、查字典美国研究</t>
+          <t>英学职沙龙刘闯/林启和</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>考研机构/转载站上岸稿，不是读研日常</t>
+          <t>学院报道转述，不是主讲人第一人称原文。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>高级翻译学院</t>
+          <t>英语学院</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1411,19 +1483,19 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>张旭校友访谈（复语班作业否决项）</t>
+          <t>北鼎/新祥旭/路灯/查字典上岸稿</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>官网风采/出色个例，口径同尚姝辰</t>
+          <t>已进半合格。考研机构稿，不充合格。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>俄语学院</t>
+          <t>高级翻译学院</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1433,12 +1505,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>赵梦雪校友会采访</t>
+          <t>张旭、文苑、尚姝辰</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>本科在黑龙江大学；北外段是硕博出色个例</t>
+          <t>已进半合格。官网/校友会风采，不充合格。</t>
         </is>
       </c>
     </row>
@@ -1450,17 +1522,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>豆瓣小语种辩护</t>
+          <t>赵梦雪校友会采访</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>学校层，未写俄语学院</t>
+          <t>已进半合格。本科黑龙江大学；出色个例。</t>
         </is>
       </c>
     </row>
@@ -1472,24 +1544,24 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>新祥旭就业率100%</t>
+          <t>豆瓣小语种辩护</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>机构推销</t>
+          <t>学校层，未写俄语学院。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>高级翻译学院</t>
+          <t>俄语学院</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1499,19 +1571,19 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>推免方案、保研指南</t>
+          <t>出国培训部俄语预科张可</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>无普通本科就读对象</t>
+          <t>预科≠俄语学院统招。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>高级翻译学院</t>
+          <t>俄语学院</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1521,12 +1593,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>尚姝辰毕业生专访、李长栓访谈</t>
+          <t>新祥旭就业率100%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>官网风采/教师，不是学生论坛自述</t>
+          <t>机构推销。</t>
         </is>
       </c>
     </row>
@@ -1538,61 +1610,61 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>北鼎法语口译在读</t>
+          <t>推免方案、保研指南</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>法语学院，不记入高翻</t>
+          <t>无普通本科就读对象。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>国际商学院</t>
+          <t>高级翻译学院</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>iMAP郑宽、国际本科评价</t>
+          <t>李长栓教师访谈</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>留学项目≠统招</t>
+          <t>老师看学生，不是学生自述；学生期末总结另条半合格。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>国际商学院</t>
+          <t>高级翻译学院</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>高顿倪子君双学位申哥大</t>
+          <t>北鼎法语口译在读邵炜</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ACCA机构学霸稿</t>
+          <t>法语学院，不记入高翻。</t>
         </is>
       </c>
     </row>
@@ -1604,24 +1676,24 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>新祥旭MIB、Reddit申请帖</t>
+          <t>iMAP郑宽、国际本科评价、冠城EAP李想</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>备考/申请，不是就读</t>
+          <t>留学/国际项目≠统招。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>国际关系学院</t>
+          <t>国际商学院</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1631,34 +1703,34 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>中青报2021级外交学、国关优秀毕业生风采</t>
+          <t>高顿倪子君双学位申哥大</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>党媒/学院风采</t>
+          <t>ACCA机构学霸稿。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>国际关系学院</t>
+          <t>国际商学院</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>本科部</t>
+          <t>研究生部</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Whever国关养老</t>
+          <t>新祥旭MIB、Reddit申请帖</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>俄语生外推，作者不在国关</t>
+          <t>备考/申请，不是就读。</t>
         </is>
       </c>
     </row>
@@ -1670,59 +1742,125 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>研究生部</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>北鼎复试/真题</t>
+          <t>中青报2021、Anette灯塔</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>机构备考</t>
+          <t>已进半合格。党媒/留学顾问约稿，不充合格。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>校级未分院</t>
+          <t>国际关系学院</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>本科部</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>就读文章1 MouradBey、7 成就你的梦想</t>
+          <t>Whever国关养老</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>未写五院之一；第7篇是付费咨询</t>
+          <t>俄语生外推，作者不在国关。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>国际关系学院</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>本科部</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>豆瓣亚运村小樱花外交科普</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>某校国关，评论像定福庄/外院，不能记北外国关。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>国际关系学院</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>研究生部</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>北鼎复试/真题</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>已进半合格。机构备考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>校级未分院</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>就读文章1 MouradBey、7 成就你的梦想</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>未写五院之一；第7篇是付费咨询</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>他院</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>就读文章2 朝鲜语、3–4 MJC</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>亚洲学院/国新，不占五院格子</t>
         </is>
@@ -1739,7 +1877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1755,54 +1893,61 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>检索日 2026-09-16（含续搜）。门槛：每院每层次 5 条「合格」第一人称就读，且尽量 3 个不同叙述者，才够做一般业余印象分析。</t>
+          <t>检索日 2026-09-16（含自述权重+在读续搜）。门槛：每院每层次 5 条「合格」第一人称就读，且尽量 3 个不同叙述者，才够做一般业余印象分析。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>合格：自称该院该层次在读/刚毕业，写课业、同学、压力、后悔等现场；非约稿、非机构广告。</t>
+          <t>文件夹目标：每部 7–10 条第一人称（合格+半合格）。公开取样不够则如实留空，不编造知乎/豆瓣正文。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>半合格：身份对得上，但正文是考研/复试/课表转载/入学后两三句。不减门槛。</t>
+          <t>合格：自称该院该层次在读/刚毕业，写课业、同学、压力、后悔等现场；非约稿、非机构广告。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Insight 采访、中青报、学院风采、高顿学霸、iMAP、北鼎/新祥旭：用户已指出可能是宣传出色个例，全部不进自述权重+。</t>
+          <t>半合格：身份对得上，但正文是考研/复试/课表转载/入学后两三句；或约稿里密课业第一人称。进夹凑条数，不减合格门槛。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>就读文章目录：只有第5、6篇 Whever 进入俄语学院本科部。第1篇未写学院，第7篇是咨询号，第2–4篇不是这五院。</t>
+          <t>Insight、中青报、张旭/文苑/尚姝辰、赵梦雪、Anette 灯塔：用户已指出可能是宣传出色个例，只进半合格。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>高翻本科部不适用。续搜补了张旭复语班作业现场，但按出色个例不进合格格；英院研究生部仍无课堂日记。</t>
+          <t>就读文章目录：只有第5、6篇 Whever 进入俄语学院本科部。第1篇未写学院，第7篇是咨询号，第2–4篇不是这五院。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>法语学院口译在读帖不记入高翻。</t>
+          <t>高翻本科部不适用。法语学院口译在读帖不记入高翻。出国培训部、iMAP、冠城EAP 不记入统招。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>豆瓣外交科普「亚运村小樱花」未确认北外国关，不进夹。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>本表在 files/论坛风云/。五个院的部级文件夹同时存在于 论坛纷纭（原取样再放置）和 论坛风云/自述权重+（过滤后）。</t>
         </is>

</xml_diff>